<commit_message>
fix: address MPO agent shutter spam and update backlog
Resolved BUG-004 related to the MPO agent spamming take-picture actions during training, leading to early episode termination. Updated backlog with new bug details and suggested fixes. Added training run logs and notebook updates for better tracking of training sessions.
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -758,7 +758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.85546875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1482,7 +1482,6 @@
           <t>todo</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>Strict JSON-driven simulation configuration loader / validator</t>
@@ -1491,6 +1490,44 @@
       <c r="H19" t="inlineStr">
         <is>
           <t>Load simulation config from one JSON source and throw hard errors for ill-defined satellite, torque policy, and camera specs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BUG-004</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>S01</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>MPO agent spams take-picture; budget early-stop blocks learning</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Notebook 08: agent fires shutter every step, exhausts capture budget, episode truncates early (early_stop_on_budget). Full-orbit rollouts never complete; learning signal collapsed. Fix: shutter action bias/exploration, reward for wasted shutters, action masking when budget low, or train-phase early-stop policy.</t>
         </is>
       </c>
     </row>

</xml_diff>